<commit_message>
Add DM Sans font files and update installed fonts configuration
- Added DM Sans font metadata in JSON format to storage/fonts.
- Created installed-fonts.json to register DM Sans with various weights.
</commit_message>
<xml_diff>
--- a/public/templates/import-siswa.xlsx
+++ b/public/templates/import-siswa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\ekskulio\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB3813DF-26A3-4955-ADB8-21DDAD292699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424FDD02-9918-485F-BBA0-A67A6E2F99AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CDC1ACF0-9087-4BBD-A3C1-E4B7A3B0C523}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t>kelas</t>
   </si>
@@ -136,6 +136,18 @@
     </r>
   </si>
   <si>
+    <t>BBA</t>
+  </si>
+  <si>
+    <t>NKA</t>
+  </si>
+  <si>
+    <t>kode_ekstrakurikuler</t>
+  </si>
+  <si>
+    <t>kelas_tujuan</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">4. </t>
     </r>
@@ -148,6 +160,32 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t xml:space="preserve">kode_ekstrakurikuler </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>diisi berdasarkan kode ekstrakurikuler yang sudah terdaftar.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">5. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>penghargaan</t>
     </r>
     <r>
@@ -162,12 +200,6 @@
     </r>
   </si>
   <si>
-    <t>BBA</t>
-  </si>
-  <si>
-    <t>NKA</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">3. </t>
     </r>
@@ -180,21 +212,18 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">kode_ekstrakurikuler </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>diisi berdasarkan kode ekstrakurikuler yang sudah terdaftar.</t>
-    </r>
-  </si>
-  <si>
-    <t>kode_ekstrakurikuler</t>
+      <t xml:space="preserve">kelas_tujuan </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>opsional, contoh: "XI RPL 1" untuk override dari "X PPLG 1".</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -226,7 +255,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -269,11 +298,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -288,13 +354,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -611,18 +683,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{865C1D33-BA53-4B78-BF39-5FAA9EC9879E}">
-  <dimension ref="A1:X6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5546875" customWidth="1"/>
-    <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" customWidth="1"/>
+    <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -633,37 +707,40 @@
         <v>0</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="G1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8"/>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="7"/>
+      <c r="X1" s="7"/>
+      <c r="Y1" s="7"/>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>12300001</v>
       </c>
@@ -673,37 +750,37 @@
       <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>2025</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="6" t="s">
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5"/>
-      <c r="U2" s="5"/>
-      <c r="V2" s="5"/>
-      <c r="W2" s="5"/>
-      <c r="X2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="S2" s="9"/>
+      <c r="T2" s="9"/>
+      <c r="U2" s="9"/>
+      <c r="V2" s="9"/>
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="10"/>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>12300002</v>
       </c>
@@ -713,37 +790,37 @@
       <c r="C3" t="s">
         <v>2</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>2024</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="6" t="s">
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="S3" s="5"/>
+      <c r="T3" s="5"/>
+      <c r="U3" s="5"/>
+      <c r="V3" s="5"/>
+      <c r="W3" s="5"/>
+      <c r="X3" s="5"/>
+      <c r="Y3" s="5"/>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>12300003</v>
       </c>
@@ -753,41 +830,53 @@
       <c r="C4" t="s">
         <v>2</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>2024</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>16</v>
       </c>
+      <c r="J4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>12300004</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>2023</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>12300005</v>
       </c>
       <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>2023</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="I2:P2"/>
-    <mergeCell ref="I3:P3"/>
-    <mergeCell ref="Q3:X3"/>
-    <mergeCell ref="I1:X1"/>
+  <mergeCells count="6">
+    <mergeCell ref="J4:Q4"/>
+    <mergeCell ref="J2:Q2"/>
+    <mergeCell ref="J3:Q3"/>
+    <mergeCell ref="R3:Y3"/>
+    <mergeCell ref="J1:Y1"/>
+    <mergeCell ref="R2:Y2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>